<commit_message>
STYLE-1: Read styles, merges, column widths, and row heights from .xlsx
</commit_message>
<xml_diff>
--- a/crates/xlsx/tests/data/fixture.xlsx
+++ b/crates/xlsx/tests/data/fixture.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Q1 Sales" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Styles" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="Rates" vbProcedure="false">Data!$C$2:$C$51</definedName>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -257,17 +258,157 @@
   </si>
   <si>
     <t xml:space="preserve">Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Styled title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hidden column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kind</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fonts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">italic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">underline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">double underline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">strike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">serif 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">red</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bold blue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fill 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fill 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fill 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fill 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">borders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">border 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">align</t>
+  </si>
+  <si>
+    <t xml:space="preserve">left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">right</t>
+  </si>
+  <si>
+    <t xml:space="preserve">top</t>
+  </si>
+  <si>
+    <t xml:space="preserve">middle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a long text that wraps inside its cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rotated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">indent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">indented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hidden row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="[$-409]#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="[$-409]0.00%"/>
+    <numFmt numFmtId="168" formatCode="[$-409]_(* #,##0_);_(* \(#,##0\);_(* \-??_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="[RED][$-409]0.00;[BLUE]\-0.00"/>
+    <numFmt numFmtId="170" formatCode="[$-409]yyyy\-mm\-dd"/>
+    <numFmt numFmtId="171" formatCode="[$-409]mmm\ d&quot;, &quot;yyyy"/>
+    <numFmt numFmtId="172" formatCode="[$-409]0.00E+00"/>
+    <numFmt numFmtId="173" formatCode="[$-409]# ?/?"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -294,21 +435,175 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u val="double"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="DejaVu Serif"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF305496"/>
+        <bgColor rgb="FF004586"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thick"/>
+      <right style="thick"/>
+      <top style="thick"/>
+      <bottom style="thick"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="dashed"/>
+      <right style="dashed"/>
+      <top style="dashed"/>
+      <bottom style="dashed"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="dotted"/>
+      <right style="dotted"/>
+      <top style="dotted"/>
+      <bottom style="dotted"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="dashDot"/>
+      <right style="dashDot"/>
+      <top style="dashDot"/>
+      <bottom style="dashDot"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFFF0000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFF0000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -337,7 +632,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -347,6 +642,154 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="45" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -359,6 +802,19 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FFCC0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -369,7 +825,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -379,28 +835,28 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0070C0"/>
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FFCC0000"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFCCCC"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -415,7 +871,7 @@
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF305496"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -611,11 +1067,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="65715860"/>
-        <c:axId val="34536254"/>
+        <c:axId val="52986256"/>
+        <c:axId val="25053903"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65715860"/>
+        <c:axId val="52986256"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -644,7 +1100,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34536254"/>
+        <c:crossAx val="25053903"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -652,7 +1108,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34536254"/>
+        <c:axId val="25053903"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -690,7 +1146,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65715860"/>
+        <c:crossAx val="52986256"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2275,4 +2731,263 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="9" min="9" style="0" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="I1" s="0" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" s="22" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="31" t="n">
+        <v>1234.5</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>3703.5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="32" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="33" t="n">
+        <v>-1234</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>-3702</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="34" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>-37.5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="35" t="n">
+        <v>46000</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>138000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="36" t="n">
+        <v>46000</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>138000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="37" t="n">
+        <v>123456</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>370368</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="38" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E8:G9"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C8:C15">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D8:D15" type="list">
+      <formula1>"yes,no"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A18" r:id="rId1" display="example"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>